<commit_message>
Update capstone project documents and Power BI files
</commit_message>
<xml_diff>
--- a/Python/Data_Metadata.xlsx
+++ b/Python/Data_Metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anitha\NIIT\Capstone Project\capstone-project-retail-tech\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC950A3D-655A-4450-A9CE-4ADCB91323EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CE912C-42D4-44DD-9C25-6B3DFB385598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -554,13 +554,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26.109375" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" customWidth="1"/>
+    <col min="6" max="6" width="17.88671875" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,7 +591,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -612,7 +617,7 @@
         <v>90000</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -638,7 +643,7 @@
         <v>19238</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -664,7 +669,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -690,7 +695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -716,7 +721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -742,7 +747,7 @@
         <v>32951</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -768,7 +773,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -794,7 +799,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -820,7 +825,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -846,7 +851,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -872,7 +877,7 @@
         <v>6068</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -898,7 +903,7 @@
         <v>6681</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -924,7 +929,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -950,7 +955,7 @@
         <v>99999</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -976,7 +981,7 @@
         <v>51895</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -1002,7 +1007,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1028,7 +1033,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1054,7 +1059,7 @@
         <v>1644</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -1080,7 +1085,7 @@
         <v>1735</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1106,7 +1111,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1132,7 +1137,7 @@
         <v>1865</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1158,7 +1163,7 @@
         <v>1702</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -1184,7 +1189,7 @@
         <v>150000</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -1210,7 +1215,7 @@
         <v>66517</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -1236,7 +1241,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -1262,7 +1267,7 @@
         <v>23534</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>39</v>
       </c>
@@ -1288,7 +1293,7 @@
         <v>4295</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -1314,7 +1319,7 @@
         <v>4844</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -1340,7 +1345,7 @@
         <v>53867</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -1366,7 +1371,7 @@
         <v>97019</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>45</v>
       </c>
@@ -1392,7 +1397,7 @@
         <v>97019</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>45</v>
       </c>
@@ -1418,7 +1423,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -1444,7 +1449,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1470,7 +1475,7 @@
         <v>1699</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -1496,7 +1501,7 @@
         <v>19238</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>50</v>
       </c>
@@ -1522,7 +1527,7 @@
         <v>128146</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -1548,7 +1553,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -1574,7 +1579,7 @@
         <v>43565</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -1600,7 +1605,7 @@
         <v>41406</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>50</v>
       </c>

</xml_diff>